<commit_message>
feat(calc): lista de precios julio v3 (definitiva) — 663 colores
vs v2: renombra 'Calacatta, Calacatta Arni' -> 'Calacatta Armi', elimina
la fila con typo 'Statuario Exra'. Cero cambios de precio. Se conservan
las correcciones de v2 (Caliza Patagonica como ARS, Negro Brasil sin
'Estandar' — ya en la fuente).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RHpNFWxWAHnD81KX3KZDvt
</commit_message>
<xml_diff>
--- a/03-product/calculadora/lista-precios-2026-07/lista-precios.xlsx
+++ b/03-product/calculadora/lista-precios-2026-07/lista-precios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sdmzi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8318AAB9-C350-4760-B202-A0B8CBFF8D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8722AFF-168C-44C6-B958-458419E9F1F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="759">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="757">
   <si>
     <t>GUIDONI QUARTZ USD MARMOLES NATURALES</t>
   </si>
@@ -1789,16 +1789,13 @@
     <t>Navona OMG</t>
   </si>
   <si>
-    <t>( A la veta, mate poro abierto)</t>
-  </si>
-  <si>
     <t>Breccia Toscana</t>
   </si>
   <si>
     <t>Breccia Vaticano</t>
   </si>
   <si>
-    <t xml:space="preserve">Calacatta, Calacatta Arni </t>
+    <t xml:space="preserve">Calacatta Armi </t>
   </si>
   <si>
     <t>Amazonite</t>
@@ -1814,9 +1811,6 @@
   </si>
   <si>
     <t xml:space="preserve">Calacatta Extra </t>
-  </si>
-  <si>
-    <t>Statuario Exra</t>
   </si>
   <si>
     <t>Statuario Michelangelo</t>
@@ -2473,10 +2467,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2489,11 +2483,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2728,7 +2722,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G881"/>
+  <dimension ref="A1:G880"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="56.42578125" customWidth="1"/>
@@ -2751,7 +2745,7 @@
         <v>899.75600000000009</v>
       </c>
       <c r="C2" s="4"/>
-      <c r="G2" s="5"/>
+      <c r="G2" s="6"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
@@ -2761,7 +2755,7 @@
         <v>899.75600000000009</v>
       </c>
       <c r="C3" s="4"/>
-      <c r="G3" s="5"/>
+      <c r="G3" s="6"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
@@ -2771,7 +2765,7 @@
         <v>899.75600000000009</v>
       </c>
       <c r="C4" s="4"/>
-      <c r="G4" s="5"/>
+      <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
@@ -2781,7 +2775,7 @@
         <v>736.1640000000001</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="G5" s="5"/>
+      <c r="G5" s="6"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -2791,7 +2785,7 @@
         <v>899.75600000000009</v>
       </c>
       <c r="C6" s="4"/>
-      <c r="G6" s="5"/>
+      <c r="G6" s="6"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
@@ -2801,7 +2795,7 @@
         <v>777.06200000000001</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="G7" s="5"/>
+      <c r="G7" s="6"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
@@ -2811,7 +2805,7 @@
         <v>531.67400000000009</v>
       </c>
       <c r="C8" s="4"/>
-      <c r="G8" s="5"/>
+      <c r="G8" s="6"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
@@ -2821,7 +2815,7 @@
         <v>531.67400000000009</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="G9" s="5"/>
+      <c r="G9" s="6"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
@@ -2831,7 +2825,7 @@
         <v>531.67400000000009</v>
       </c>
       <c r="C10" s="4"/>
-      <c r="G10" s="5"/>
+      <c r="G10" s="6"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
@@ -2841,7 +2835,7 @@
         <v>633.9190000000001</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="G11" s="5"/>
+      <c r="G11" s="6"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
@@ -2851,7 +2845,7 @@
         <v>654.36800000000005</v>
       </c>
       <c r="C12" s="4"/>
-      <c r="G12" s="5"/>
+      <c r="G12" s="6"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
@@ -2861,7 +2855,7 @@
         <v>736.1640000000001</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="G13" s="5"/>
+      <c r="G13" s="6"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
@@ -2871,7 +2865,7 @@
         <v>736.1640000000001</v>
       </c>
       <c r="C14" s="4"/>
-      <c r="G14" s="5"/>
+      <c r="G14" s="6"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
@@ -2881,7 +2875,7 @@
         <v>654.36800000000005</v>
       </c>
       <c r="C15" s="4"/>
-      <c r="G15" s="5"/>
+      <c r="G15" s="6"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
@@ -2891,7 +2885,7 @@
         <v>1226.94</v>
       </c>
       <c r="C16" s="4"/>
-      <c r="G16" s="5"/>
+      <c r="G16" s="6"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
@@ -2901,7 +2895,7 @@
         <v>654.36800000000005</v>
       </c>
       <c r="C17" s="4"/>
-      <c r="G17" s="5"/>
+      <c r="G17" s="6"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
@@ -2911,7 +2905,7 @@
         <v>715.71500000000015</v>
       </c>
       <c r="C18" s="4"/>
-      <c r="G18" s="5"/>
+      <c r="G18" s="6"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
@@ -2921,7 +2915,7 @@
         <v>715.71500000000015</v>
       </c>
       <c r="C19" s="4"/>
-      <c r="G19" s="5"/>
+      <c r="G19" s="6"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
@@ -2931,7 +2925,7 @@
         <v>756.61300000000006</v>
       </c>
       <c r="C20" s="4"/>
-      <c r="G20" s="5"/>
+      <c r="G20" s="6"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
@@ -2941,7 +2935,7 @@
         <v>756.61300000000006</v>
       </c>
       <c r="C21" s="4"/>
-      <c r="G21" s="5"/>
+      <c r="G21" s="6"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
@@ -2951,7 +2945,7 @@
         <v>756.61300000000006</v>
       </c>
       <c r="C22" s="4"/>
-      <c r="G22" s="5"/>
+      <c r="G22" s="6"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
@@ -2961,7 +2955,7 @@
         <v>1226.94</v>
       </c>
       <c r="C23" s="4"/>
-      <c r="G23" s="5"/>
+      <c r="G23" s="6"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
@@ -2971,7 +2965,7 @@
         <v>899.75600000000009</v>
       </c>
       <c r="C24" s="4"/>
-      <c r="G24" s="5"/>
+      <c r="G24" s="6"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
@@ -2981,7 +2975,7 @@
         <v>756.61300000000006</v>
       </c>
       <c r="C25" s="4"/>
-      <c r="G25" s="5"/>
+      <c r="G25" s="6"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
@@ -2991,7 +2985,7 @@
         <v>756.61300000000006</v>
       </c>
       <c r="C26" s="4"/>
-      <c r="G26" s="5"/>
+      <c r="G26" s="6"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
@@ -3001,7 +2995,7 @@
         <v>613.47</v>
       </c>
       <c r="C27" s="4"/>
-      <c r="G27" s="5"/>
+      <c r="G27" s="6"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
@@ -3011,7 +3005,7 @@
         <v>1431.4300000000003</v>
       </c>
       <c r="C28" s="4"/>
-      <c r="G28" s="5"/>
+      <c r="G28" s="6"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
@@ -3159,7 +3153,7 @@
       <c r="B47" s="2"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A48" s="13" t="s">
+      <c r="A48" s="14" t="s">
         <v>45</v>
       </c>
       <c r="B48" s="2"/>
@@ -3189,7 +3183,7 @@
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A52" s="14" t="s">
+      <c r="A52" s="15" t="s">
         <v>49</v>
       </c>
       <c r="B52" s="2"/>
@@ -3219,7 +3213,7 @@
       <c r="G55" s="11"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A56" s="13" t="s">
+      <c r="A56" s="14" t="s">
         <v>52</v>
       </c>
       <c r="B56" s="9"/>
@@ -3228,7 +3222,7 @@
       <c r="G56" s="11"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A57" s="14" t="s">
+      <c r="A57" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B57" s="9"/>
@@ -3297,7 +3291,7 @@
       <c r="B66" s="2"/>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A67" s="13" t="s">
+      <c r="A67" s="14" t="s">
         <v>61</v>
       </c>
       <c r="B67" s="2"/>
@@ -3574,7 +3568,7 @@
       <c r="B103" s="2"/>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A104" s="13" t="s">
+      <c r="A104" s="14" t="s">
         <v>97</v>
       </c>
       <c r="B104" s="2"/>
@@ -3771,7 +3765,7 @@
       <c r="B131" s="2">
         <v>593.125</v>
       </c>
-      <c r="C131" s="6"/>
+      <c r="C131" s="5"/>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B132" s="2"/>
@@ -4231,7 +4225,7 @@
       <c r="B194" s="2"/>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A195" s="13" t="s">
+      <c r="A195" s="14" t="s">
         <v>177</v>
       </c>
       <c r="B195" s="2">
@@ -4282,7 +4276,7 @@
       <c r="A201" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="B201" s="15">
+      <c r="B201" s="13">
         <v>660.66000000000008</v>
       </c>
     </row>
@@ -4306,7 +4300,7 @@
       <c r="A204" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="B204" s="15">
+      <c r="B204" s="13">
         <v>660.66000000000008</v>
       </c>
     </row>
@@ -4378,7 +4372,7 @@
       <c r="A213" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="B213" s="15">
+      <c r="B213" s="13">
         <v>660.66000000000008</v>
       </c>
     </row>
@@ -4418,7 +4412,7 @@
       <c r="A218" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="B218" s="15">
+      <c r="B218" s="13">
         <v>660.66000000000008</v>
       </c>
     </row>
@@ -4426,7 +4420,7 @@
       <c r="A219" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="B219" s="15">
+      <c r="B219" s="13">
         <v>660.66000000000008</v>
       </c>
     </row>
@@ -4434,7 +4428,7 @@
       <c r="A220" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="B220" s="15">
+      <c r="B220" s="13">
         <v>707.85</v>
       </c>
     </row>
@@ -4640,7 +4634,7 @@
       <c r="B248" s="2"/>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A249" s="13" t="s">
+      <c r="A249" s="14" t="s">
         <v>226</v>
       </c>
       <c r="B249" s="2"/>
@@ -4662,7 +4656,7 @@
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A252" s="13" t="s">
+      <c r="A252" s="14" t="s">
         <v>229</v>
       </c>
       <c r="B252" s="2"/>
@@ -4724,7 +4718,7 @@
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A260" s="13" t="s">
+      <c r="A260" s="14" t="s">
         <v>237</v>
       </c>
       <c r="B260" s="2"/>
@@ -4810,7 +4804,7 @@
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A271" s="13" t="s">
+      <c r="A271" s="14" t="s">
         <v>248</v>
       </c>
       <c r="B271" s="2"/>
@@ -4935,11 +4929,11 @@
       <c r="B287" s="2"/>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A288" s="13" t="s">
+      <c r="A288" s="14" t="s">
         <v>264</v>
       </c>
       <c r="B288" s="2"/>
-      <c r="G288" s="13"/>
+      <c r="G288" s="14"/>
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A289" s="3" t="s">
@@ -4969,11 +4963,11 @@
       <c r="B292" s="2"/>
     </row>
     <row r="293" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A293" s="13" t="s">
+      <c r="A293" s="14" t="s">
         <v>268</v>
       </c>
       <c r="B293" s="2"/>
-      <c r="G293" s="13"/>
+      <c r="G293" s="14"/>
     </row>
     <row r="294" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A294" s="3" t="s">
@@ -5027,11 +5021,11 @@
       <c r="B300" s="2"/>
     </row>
     <row r="301" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A301" s="13" t="s">
+      <c r="A301" s="14" t="s">
         <v>275</v>
       </c>
       <c r="B301" s="2"/>
-      <c r="G301" s="13"/>
+      <c r="G301" s="14"/>
     </row>
     <row r="302" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A302" s="3" t="s">
@@ -5098,11 +5092,11 @@
       </c>
     </row>
     <row r="310" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A310" s="13" t="s">
+      <c r="A310" s="14" t="s">
         <v>248</v>
       </c>
       <c r="B310" s="2"/>
-      <c r="G310" s="13"/>
+      <c r="G310" s="14"/>
     </row>
     <row r="311" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A311" s="3" t="s">
@@ -5156,11 +5150,11 @@
       <c r="B317" s="2"/>
     </row>
     <row r="318" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A318" s="13" t="s">
+      <c r="A318" s="14" t="s">
         <v>290</v>
       </c>
       <c r="B318" s="2"/>
-      <c r="G318" s="13"/>
+      <c r="G318" s="14"/>
     </row>
     <row r="319" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A319" s="3" t="s">
@@ -5214,11 +5208,11 @@
       <c r="B325" s="2"/>
     </row>
     <row r="326" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A326" s="13" t="s">
+      <c r="A326" s="14" t="s">
         <v>297</v>
       </c>
       <c r="B326" s="2"/>
-      <c r="G326" s="13"/>
+      <c r="G326" s="14"/>
     </row>
     <row r="327" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A327" s="3" t="s">
@@ -5280,11 +5274,11 @@
       <c r="B334" s="2"/>
     </row>
     <row r="335" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A335" s="13" t="s">
+      <c r="A335" s="14" t="s">
         <v>305</v>
       </c>
       <c r="B335" s="2"/>
-      <c r="G335" s="13"/>
+      <c r="G335" s="14"/>
     </row>
     <row r="336" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B336" s="9"/>
@@ -5317,11 +5311,11 @@
       <c r="B340" s="2"/>
     </row>
     <row r="341" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A341" s="13" t="s">
+      <c r="A341" s="14" t="s">
         <v>309</v>
       </c>
       <c r="B341" s="2"/>
-      <c r="G341" s="13"/>
+      <c r="G341" s="14"/>
     </row>
     <row r="342" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A342" s="3" t="s">
@@ -5362,7 +5356,7 @@
       <c r="B347" s="2"/>
     </row>
     <row r="348" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A348" s="13" t="s">
+      <c r="A348" s="14" t="s">
         <v>264</v>
       </c>
       <c r="B348" s="2"/>
@@ -5443,7 +5437,7 @@
       <c r="B358" s="2"/>
     </row>
     <row r="359" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A359" s="13" t="s">
+      <c r="A359" s="14" t="s">
         <v>268</v>
       </c>
       <c r="B359" s="2"/>
@@ -5548,7 +5542,7 @@
       <c r="B372" s="2"/>
     </row>
     <row r="373" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A373" s="13" t="s">
+      <c r="A373" s="14" t="s">
         <v>237</v>
       </c>
       <c r="B373" s="2"/>
@@ -5661,7 +5655,7 @@
       <c r="B387" s="2"/>
     </row>
     <row r="388" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A388" s="13" t="s">
+      <c r="A388" s="14" t="s">
         <v>248</v>
       </c>
       <c r="B388" s="2"/>
@@ -5710,7 +5704,7 @@
       <c r="B394" s="2"/>
     </row>
     <row r="395" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A395" s="13" t="s">
+      <c r="A395" s="14" t="s">
         <v>290</v>
       </c>
       <c r="B395" s="2"/>
@@ -5757,11 +5751,11 @@
       <c r="B401" s="2"/>
     </row>
     <row r="402" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A402" s="13"/>
+      <c r="A402" s="14"/>
       <c r="B402" s="2"/>
     </row>
     <row r="403" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A403" s="13" t="s">
+      <c r="A403" s="14" t="s">
         <v>264</v>
       </c>
       <c r="B403" s="2"/>
@@ -5858,7 +5852,7 @@
       <c r="B415" s="2"/>
     </row>
     <row r="416" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A416" s="13" t="s">
+      <c r="A416" s="14" t="s">
         <v>369</v>
       </c>
       <c r="B416" s="2"/>
@@ -5923,7 +5917,7 @@
       <c r="B424" s="2"/>
     </row>
     <row r="425" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A425" s="13" t="s">
+      <c r="A425" s="14" t="s">
         <v>52</v>
       </c>
       <c r="B425" s="2"/>
@@ -5972,7 +5966,7 @@
       <c r="B431" s="2"/>
     </row>
     <row r="432" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A432" s="13" t="s">
+      <c r="A432" s="14" t="s">
         <v>382</v>
       </c>
       <c r="B432" s="2"/>
@@ -6027,7 +6021,7 @@
       <c r="B439" s="2"/>
     </row>
     <row r="440" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A440" s="13" t="s">
+      <c r="A440" s="14" t="s">
         <v>226</v>
       </c>
       <c r="B440" s="2"/>
@@ -6129,7 +6123,7 @@
       </c>
     </row>
     <row r="453" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A453" s="13" t="s">
+      <c r="A453" s="14" t="s">
         <v>229</v>
       </c>
       <c r="B453" s="2"/>
@@ -6213,7 +6207,7 @@
       <c r="B464" s="2"/>
     </row>
     <row r="465" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A465" s="13" t="s">
+      <c r="A465" s="14" t="s">
         <v>275</v>
       </c>
       <c r="B465" s="2"/>
@@ -6290,7 +6284,7 @@
       <c r="B475" s="2"/>
     </row>
     <row r="476" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A476" s="13" t="s">
+      <c r="A476" s="14" t="s">
         <v>248</v>
       </c>
       <c r="B476" s="2"/>
@@ -6352,7 +6346,7 @@
       </c>
     </row>
     <row r="484" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A484" s="13" t="s">
+      <c r="A484" s="14" t="s">
         <v>290</v>
       </c>
       <c r="B484" s="2"/>
@@ -6423,7 +6417,7 @@
       </c>
     </row>
     <row r="493" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A493" s="13" t="s">
+      <c r="A493" s="14" t="s">
         <v>297</v>
       </c>
       <c r="B493" s="2"/>
@@ -7537,7 +7531,7 @@
       <c r="B634" s="2"/>
     </row>
     <row r="635" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A635" s="13" t="s">
+      <c r="A635" s="14" t="s">
         <v>369</v>
       </c>
       <c r="B635" s="2"/>
@@ -7551,23 +7545,20 @@
       </c>
     </row>
     <row r="637" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A637" s="3" t="s">
-        <v>565</v>
-      </c>
       <c r="B637" s="2"/>
     </row>
     <row r="638" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B638" s="2"/>
     </row>
     <row r="639" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A639" s="13" t="s">
+      <c r="A639" s="14" t="s">
         <v>52</v>
       </c>
       <c r="B639" s="2"/>
     </row>
     <row r="640" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A640" s="3" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B640" s="2">
         <v>2905.5</v>
@@ -7575,7 +7566,7 @@
     </row>
     <row r="641" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A641" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B641" s="2">
         <v>2905.5</v>
@@ -7583,7 +7574,7 @@
     </row>
     <row r="642" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A642" s="3" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B642" s="2">
         <v>2905.5</v>
@@ -7598,14 +7589,14 @@
       </c>
     </row>
     <row r="644" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A644" s="13" t="s">
+      <c r="A644" s="14" t="s">
         <v>382</v>
       </c>
       <c r="B644" s="2"/>
     </row>
     <row r="645" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A645" s="3" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B645" s="2">
         <v>3250</v>
@@ -7613,7 +7604,7 @@
     </row>
     <row r="646" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A646" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B646" s="2">
         <v>3250</v>
@@ -7621,7 +7612,7 @@
     </row>
     <row r="647" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A647" s="3" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B647" s="2">
         <v>3250</v>
@@ -7631,14 +7622,14 @@
       <c r="B648" s="2"/>
     </row>
     <row r="649" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A649" s="13" t="s">
-        <v>572</v>
+      <c r="A649" s="14" t="s">
+        <v>571</v>
       </c>
       <c r="B649" s="2"/>
     </row>
     <row r="650" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A650" s="3" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B650" s="2">
         <v>3859.375</v>
@@ -7646,32 +7637,32 @@
     </row>
     <row r="651" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A651" s="3" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B651" s="2">
         <v>3859.375</v>
       </c>
     </row>
     <row r="652" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A652" s="3" t="s">
+      <c r="B652" s="2"/>
+    </row>
+    <row r="653" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A653" s="14" t="s">
+        <v>574</v>
+      </c>
+      <c r="B653" s="2"/>
+    </row>
+    <row r="654" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A654" s="3" t="s">
         <v>575</v>
       </c>
-      <c r="B652" s="2">
-        <v>3859.375</v>
-      </c>
-    </row>
-    <row r="653" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B653" s="2"/>
-    </row>
-    <row r="654" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A654" s="13" t="s">
-        <v>576</v>
-      </c>
-      <c r="B654" s="2"/>
+      <c r="B654" s="2">
+        <v>4671.875</v>
+      </c>
     </row>
     <row r="655" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A655" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B655" s="2">
         <v>4671.875</v>
@@ -7679,7 +7670,7 @@
     </row>
     <row r="656" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A656" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B656" s="2">
         <v>4671.875</v>
@@ -7687,63 +7678,63 @@
     </row>
     <row r="657" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A657" s="3" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B657" s="2">
         <v>4671.875</v>
       </c>
     </row>
     <row r="658" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A658" s="3" t="s">
+      <c r="B658" s="2"/>
+    </row>
+    <row r="659" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A659" s="14" t="s">
+        <v>579</v>
+      </c>
+      <c r="B659" s="2"/>
+    </row>
+    <row r="660" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A660" s="3" t="s">
         <v>580</v>
       </c>
-      <c r="B658" s="2">
-        <v>4671.875</v>
-      </c>
-    </row>
-    <row r="659" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B659" s="2"/>
-    </row>
-    <row r="660" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A660" s="13" t="s">
-        <v>581</v>
-      </c>
-      <c r="B660" s="2"/>
+      <c r="B660" s="2">
+        <v>7312.5</v>
+      </c>
     </row>
     <row r="661" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A661" s="3" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B661" s="2">
         <v>7312.5</v>
       </c>
     </row>
     <row r="662" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A662" s="3" t="s">
+      <c r="B662" s="2"/>
+    </row>
+    <row r="663" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A663" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="B663" s="2"/>
+    </row>
+    <row r="664" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A664" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="B664" s="2"/>
+    </row>
+    <row r="665" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A665" s="3" t="s">
         <v>583</v>
       </c>
-      <c r="B662" s="2">
-        <v>7312.5</v>
-      </c>
-    </row>
-    <row r="663" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B663" s="2"/>
-    </row>
-    <row r="664" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A664" s="1" t="s">
-        <v>584</v>
-      </c>
-      <c r="B664" s="2"/>
-    </row>
-    <row r="665" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A665" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="B665" s="2"/>
+      <c r="B665" s="2">
+        <v>406.25</v>
+      </c>
     </row>
     <row r="666" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A666" s="3" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B666" s="2">
         <v>406.25</v>
@@ -7751,7 +7742,7 @@
     </row>
     <row r="667" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A667" s="3" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B667" s="2">
         <v>406.25</v>
@@ -7759,7 +7750,7 @@
     </row>
     <row r="668" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A668" s="3" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B668" s="2">
         <v>406.25</v>
@@ -7767,7 +7758,7 @@
     </row>
     <row r="669" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A669" s="3" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B669" s="2">
         <v>406.25</v>
@@ -7775,7 +7766,7 @@
     </row>
     <row r="670" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A670" s="3" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B670" s="2">
         <v>406.25</v>
@@ -7783,7 +7774,7 @@
     </row>
     <row r="671" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A671" s="3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B671" s="2">
         <v>406.25</v>
@@ -7791,32 +7782,32 @@
     </row>
     <row r="672" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A672" s="3" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B672" s="2">
         <v>406.25</v>
       </c>
     </row>
     <row r="673" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A673" s="3" t="s">
-        <v>592</v>
-      </c>
-      <c r="B673" s="2">
-        <v>406.25</v>
-      </c>
+      <c r="B673" s="2"/>
     </row>
     <row r="674" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A674" s="14" t="s">
+        <v>268</v>
+      </c>
       <c r="B674" s="2"/>
     </row>
     <row r="675" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A675" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="B675" s="2"/>
+      <c r="A675" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="B675" s="2">
+        <v>549.25</v>
+      </c>
     </row>
     <row r="676" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A676" s="3" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B676" s="2">
         <v>549.25</v>
@@ -7824,7 +7815,7 @@
     </row>
     <row r="677" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A677" s="3" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B677" s="2">
         <v>549.25</v>
@@ -7832,7 +7823,7 @@
     </row>
     <row r="678" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A678" s="3" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B678" s="2">
         <v>549.25</v>
@@ -7840,7 +7831,7 @@
     </row>
     <row r="679" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A679" s="3" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B679" s="2">
         <v>549.25</v>
@@ -7848,7 +7839,7 @@
     </row>
     <row r="680" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A680" s="3" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B680" s="2">
         <v>549.25</v>
@@ -7856,7 +7847,7 @@
     </row>
     <row r="681" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A681" s="3" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B681" s="2">
         <v>549.25</v>
@@ -7864,7 +7855,7 @@
     </row>
     <row r="682" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A682" s="3" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B682" s="2">
         <v>549.25</v>
@@ -7872,7 +7863,7 @@
     </row>
     <row r="683" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A683" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B683" s="2">
         <v>549.25</v>
@@ -7880,32 +7871,32 @@
     </row>
     <row r="684" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A684" s="3" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B684" s="2">
         <v>549.25</v>
       </c>
     </row>
     <row r="685" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A685" s="3" t="s">
+      <c r="B685" s="2"/>
+    </row>
+    <row r="686" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A686" s="14" t="s">
+        <v>601</v>
+      </c>
+      <c r="B686" s="2"/>
+    </row>
+    <row r="687" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A687" s="3" t="s">
         <v>602</v>
       </c>
-      <c r="B685" s="2">
-        <v>549.25</v>
-      </c>
-    </row>
-    <row r="686" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B686" s="2"/>
-    </row>
-    <row r="687" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A687" s="13" t="s">
-        <v>603</v>
-      </c>
-      <c r="B687" s="2"/>
+      <c r="B687" s="2">
+        <v>690.625</v>
+      </c>
     </row>
     <row r="688" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A688" s="3" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B688" s="2">
         <v>690.625</v>
@@ -7913,7 +7904,7 @@
     </row>
     <row r="689" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A689" s="3" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B689" s="2">
         <v>690.625</v>
@@ -7921,7 +7912,7 @@
     </row>
     <row r="690" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A690" s="3" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B690" s="2">
         <v>690.625</v>
@@ -7929,7 +7920,7 @@
     </row>
     <row r="691" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A691" s="3" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B691" s="2">
         <v>690.625</v>
@@ -7937,7 +7928,7 @@
     </row>
     <row r="692" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A692" s="3" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B692" s="2">
         <v>690.625</v>
@@ -7945,7 +7936,7 @@
     </row>
     <row r="693" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A693" s="3" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B693" s="2">
         <v>690.625</v>
@@ -7953,7 +7944,7 @@
     </row>
     <row r="694" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A694" s="3" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B694" s="2">
         <v>690.625</v>
@@ -7961,7 +7952,7 @@
     </row>
     <row r="695" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A695" s="3" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B695" s="2">
         <v>690.625</v>
@@ -7969,7 +7960,7 @@
     </row>
     <row r="696" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A696" s="3" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B696" s="2">
         <v>690.625</v>
@@ -7977,7 +7968,7 @@
     </row>
     <row r="697" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A697" s="3" t="s">
-        <v>613</v>
+        <v>172</v>
       </c>
       <c r="B697" s="2">
         <v>690.625</v>
@@ -7985,7 +7976,7 @@
     </row>
     <row r="698" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A698" s="3" t="s">
-        <v>172</v>
+        <v>612</v>
       </c>
       <c r="B698" s="2">
         <v>690.625</v>
@@ -7993,7 +7984,7 @@
     </row>
     <row r="699" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A699" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B699" s="2">
         <v>690.625</v>
@@ -8001,7 +7992,7 @@
     </row>
     <row r="700" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A700" s="3" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B700" s="2">
         <v>690.625</v>
@@ -8009,7 +8000,7 @@
     </row>
     <row r="701" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A701" s="3" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B701" s="2">
         <v>690.625</v>
@@ -8017,7 +8008,7 @@
     </row>
     <row r="702" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A702" s="3" t="s">
-        <v>617</v>
+        <v>507</v>
       </c>
       <c r="B702" s="2">
         <v>690.625</v>
@@ -8025,32 +8016,32 @@
     </row>
     <row r="703" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A703" s="3" t="s">
-        <v>507</v>
+        <v>616</v>
       </c>
       <c r="B703" s="2">
         <v>690.625</v>
       </c>
     </row>
     <row r="704" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A704" s="3" t="s">
-        <v>618</v>
-      </c>
-      <c r="B704" s="2">
-        <v>690.625</v>
-      </c>
+      <c r="B704" s="2"/>
     </row>
     <row r="705" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A705" s="14" t="s">
+        <v>382</v>
+      </c>
       <c r="B705" s="2"/>
     </row>
     <row r="706" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A706" s="13" t="s">
-        <v>382</v>
-      </c>
-      <c r="B706" s="2"/>
+      <c r="A706" s="3" t="s">
+        <v>617</v>
+      </c>
+      <c r="B706" s="2">
+        <v>812.5</v>
+      </c>
     </row>
     <row r="707" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A707" s="3" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B707" s="2">
         <v>812.5</v>
@@ -8058,7 +8049,7 @@
     </row>
     <row r="708" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A708" s="3" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B708" s="2">
         <v>812.5</v>
@@ -8066,7 +8057,7 @@
     </row>
     <row r="709" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A709" s="3" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B709" s="2">
         <v>812.5</v>
@@ -8074,7 +8065,7 @@
     </row>
     <row r="710" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A710" s="3" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B710" s="2">
         <v>812.5</v>
@@ -8082,7 +8073,7 @@
     </row>
     <row r="711" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A711" s="3" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B711" s="2">
         <v>812.5</v>
@@ -8090,7 +8081,7 @@
     </row>
     <row r="712" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A712" s="3" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B712" s="2">
         <v>812.5</v>
@@ -8098,7 +8089,7 @@
     </row>
     <row r="713" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A713" s="3" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B713" s="2">
         <v>812.5</v>
@@ -8106,7 +8097,7 @@
     </row>
     <row r="714" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A714" s="3" t="s">
-        <v>626</v>
+        <v>168</v>
       </c>
       <c r="B714" s="2">
         <v>812.5</v>
@@ -8114,7 +8105,7 @@
     </row>
     <row r="715" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A715" s="3" t="s">
-        <v>168</v>
+        <v>625</v>
       </c>
       <c r="B715" s="2">
         <v>812.5</v>
@@ -8122,7 +8113,7 @@
     </row>
     <row r="716" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A716" s="3" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B716" s="2">
         <v>812.5</v>
@@ -8130,32 +8121,32 @@
     </row>
     <row r="717" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A717" s="3" t="s">
-        <v>628</v>
+        <v>164</v>
       </c>
       <c r="B717" s="2">
         <v>812.5</v>
       </c>
     </row>
     <row r="718" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A718" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="B718" s="2">
-        <v>812.5</v>
-      </c>
+      <c r="B718" s="2"/>
     </row>
     <row r="719" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A719" s="14" t="s">
+        <v>627</v>
+      </c>
       <c r="B719" s="2"/>
     </row>
     <row r="720" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A720" s="13" t="s">
-        <v>629</v>
-      </c>
-      <c r="B720" s="2"/>
+      <c r="A720" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="B720" s="2">
+        <v>1218.75</v>
+      </c>
     </row>
     <row r="721" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A721" s="3" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B721" s="2">
         <v>1218.75</v>
@@ -8163,7 +8154,7 @@
     </row>
     <row r="722" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A722" s="3" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B722" s="2">
         <v>1218.75</v>
@@ -8171,7 +8162,7 @@
     </row>
     <row r="723" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A723" s="3" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B723" s="2">
         <v>1218.75</v>
@@ -8179,7 +8170,7 @@
     </row>
     <row r="724" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A724" s="3" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B724" s="2">
         <v>1218.75</v>
@@ -8187,7 +8178,7 @@
     </row>
     <row r="725" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A725" s="3" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B725" s="2">
         <v>1218.75</v>
@@ -8195,7 +8186,7 @@
     </row>
     <row r="726" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A726" s="3" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B726" s="2">
         <v>1218.75</v>
@@ -8203,7 +8194,7 @@
     </row>
     <row r="727" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A727" s="3" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B727" s="2">
         <v>1218.75</v>
@@ -8211,7 +8202,7 @@
     </row>
     <row r="728" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A728" s="3" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B728" s="2">
         <v>1218.75</v>
@@ -8219,7 +8210,7 @@
     </row>
     <row r="729" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A729" s="3" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B729" s="2">
         <v>1218.75</v>
@@ -8227,7 +8218,7 @@
     </row>
     <row r="730" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A730" s="3" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B730" s="2">
         <v>1218.75</v>
@@ -8235,7 +8226,7 @@
     </row>
     <row r="731" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A731" s="3" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B731" s="2">
         <v>1218.75</v>
@@ -8243,7 +8234,7 @@
     </row>
     <row r="732" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A732" s="3" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B732" s="2">
         <v>1218.75</v>
@@ -8251,7 +8242,7 @@
     </row>
     <row r="733" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A733" s="3" t="s">
-        <v>642</v>
+        <v>159</v>
       </c>
       <c r="B733" s="2">
         <v>1218.75</v>
@@ -8259,32 +8250,32 @@
     </row>
     <row r="734" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A734" s="3" t="s">
-        <v>159</v>
+        <v>641</v>
       </c>
       <c r="B734" s="2">
         <v>1218.75</v>
       </c>
     </row>
     <row r="735" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A735" s="3" t="s">
+      <c r="B735" s="2"/>
+    </row>
+    <row r="736" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A736" s="14" t="s">
+        <v>642</v>
+      </c>
+      <c r="B736" s="2"/>
+    </row>
+    <row r="737" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A737" s="3" t="s">
         <v>643</v>
       </c>
-      <c r="B735" s="2">
-        <v>1218.75</v>
-      </c>
-    </row>
-    <row r="736" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B736" s="2"/>
-    </row>
-    <row r="737" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A737" s="13" t="s">
-        <v>644</v>
-      </c>
-      <c r="B737" s="2"/>
+      <c r="B737" s="2">
+        <v>1828.125</v>
+      </c>
     </row>
     <row r="738" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A738" s="3" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B738" s="2">
         <v>1828.125</v>
@@ -8292,7 +8283,7 @@
     </row>
     <row r="739" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A739" s="3" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B739" s="2">
         <v>1828.125</v>
@@ -8300,7 +8291,7 @@
     </row>
     <row r="740" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A740" s="3" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B740" s="2">
         <v>1828.125</v>
@@ -8308,7 +8299,7 @@
     </row>
     <row r="741" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A741" s="3" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B741" s="2">
         <v>1828.125</v>
@@ -8316,7 +8307,7 @@
     </row>
     <row r="742" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A742" s="3" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B742" s="2">
         <v>1828.125</v>
@@ -8324,7 +8315,7 @@
     </row>
     <row r="743" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A743" s="3" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B743" s="2">
         <v>1828.125</v>
@@ -8332,7 +8323,7 @@
     </row>
     <row r="744" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A744" s="3" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B744" s="2">
         <v>1828.125</v>
@@ -8340,7 +8331,7 @@
     </row>
     <row r="745" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A745" s="3" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B745" s="2">
         <v>1828.125</v>
@@ -8348,7 +8339,7 @@
     </row>
     <row r="746" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A746" s="3" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B746" s="2">
         <v>1828.125</v>
@@ -8356,7 +8347,7 @@
     </row>
     <row r="747" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A747" s="3" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B747" s="2">
         <v>1828.125</v>
@@ -8364,7 +8355,7 @@
     </row>
     <row r="748" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A748" s="3" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B748" s="2">
         <v>1828.125</v>
@@ -8372,7 +8363,7 @@
     </row>
     <row r="749" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A749" s="3" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B749" s="2">
         <v>1828.125</v>
@@ -8380,7 +8371,7 @@
     </row>
     <row r="750" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A750" s="3" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B750" s="2">
         <v>1828.125</v>
@@ -8388,56 +8379,56 @@
     </row>
     <row r="751" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A751" s="3" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B751" s="2">
         <v>1828.125</v>
       </c>
     </row>
     <row r="752" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A752" s="3" t="s">
+      <c r="B752" s="2"/>
+    </row>
+    <row r="753" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A753" s="1" t="s">
+        <v>658</v>
+      </c>
+      <c r="B753" s="2"/>
+    </row>
+    <row r="754" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A754" s="3" t="s">
         <v>659</v>
       </c>
-      <c r="B752" s="2">
-        <v>1828.125</v>
-      </c>
-    </row>
-    <row r="753" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B753" s="2"/>
-    </row>
-    <row r="754" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A754" s="1" t="s">
-        <v>660</v>
-      </c>
-      <c r="B754" s="2"/>
+      <c r="B754" s="2">
+        <v>812.5</v>
+      </c>
     </row>
     <row r="755" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A755" s="3" t="s">
-        <v>661</v>
+        <v>643</v>
       </c>
       <c r="B755" s="2">
-        <v>812.5</v>
+        <v>1828.125</v>
       </c>
     </row>
     <row r="756" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A756" s="3" t="s">
-        <v>645</v>
+        <v>660</v>
       </c>
       <c r="B756" s="2">
-        <v>1828.125</v>
+        <v>1218.75</v>
       </c>
     </row>
     <row r="757" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A757" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B757" s="2">
-        <v>1218.75</v>
+        <v>2096.25</v>
       </c>
     </row>
     <row r="758" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A758" s="3" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B758" s="2">
         <v>2096.25</v>
@@ -8445,90 +8436,90 @@
     </row>
     <row r="759" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A759" s="3" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B759" s="2">
-        <v>2096.25</v>
+        <v>3152.5</v>
       </c>
     </row>
     <row r="760" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A760" s="3" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B760" s="2">
-        <v>3152.5</v>
+        <v>1218.75</v>
       </c>
     </row>
     <row r="761" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A761" s="3" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B761" s="2">
-        <v>1218.75</v>
+        <v>1828.125</v>
       </c>
     </row>
     <row r="762" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A762" s="3" t="s">
-        <v>667</v>
-      </c>
-      <c r="B762" s="2">
-        <v>1828.125</v>
-      </c>
+      <c r="B762" s="2"/>
     </row>
     <row r="763" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B763" s="2"/>
     </row>
     <row r="764" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A764" s="19" t="s">
+        <v>666</v>
+      </c>
       <c r="B764" s="2"/>
     </row>
     <row r="765" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A765" s="19" t="s">
-        <v>668</v>
-      </c>
-      <c r="B765" s="2"/>
+      <c r="A765" s="3" t="s">
+        <v>667</v>
+      </c>
+      <c r="B765" s="2">
+        <v>786.5</v>
+      </c>
     </row>
     <row r="766" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A766" s="3" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B766" s="2">
-        <v>786.5</v>
+        <v>1085.3700000000001</v>
       </c>
     </row>
     <row r="767" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A767" s="3" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B767" s="2">
         <v>1085.3700000000001</v>
       </c>
     </row>
     <row r="768" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A768" s="3" t="s">
+      <c r="B768" s="2"/>
+    </row>
+    <row r="769" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A769" s="1" t="s">
+        <v>670</v>
+      </c>
+      <c r="B769" s="2"/>
+    </row>
+    <row r="770" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A770" s="14" t="s">
         <v>671</v>
       </c>
-      <c r="B768" s="2">
-        <v>1085.3700000000001</v>
-      </c>
-    </row>
-    <row r="769" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B769" s="2"/>
-    </row>
-    <row r="770" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A770" s="1" t="s">
+      <c r="B770" s="2"/>
+    </row>
+    <row r="771" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A771" s="3" t="s">
         <v>672</v>
       </c>
-      <c r="B770" s="2"/>
-    </row>
-    <row r="771" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A771" s="13" t="s">
-        <v>673</v>
-      </c>
-      <c r="B771" s="2"/>
+      <c r="B771" s="2">
+        <v>446.875</v>
+      </c>
     </row>
     <row r="772" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A772" s="3" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="B772" s="2">
         <v>446.875</v>
@@ -8536,7 +8527,7 @@
     </row>
     <row r="773" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A773" s="3" t="s">
-        <v>675</v>
+        <v>636</v>
       </c>
       <c r="B773" s="2">
         <v>446.875</v>
@@ -8544,32 +8535,32 @@
     </row>
     <row r="774" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A774" s="3" t="s">
-        <v>638</v>
+        <v>674</v>
       </c>
       <c r="B774" s="2">
         <v>446.875</v>
       </c>
     </row>
     <row r="775" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A775" s="3" t="s">
+      <c r="B775" s="2"/>
+    </row>
+    <row r="776" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A776" s="14" t="s">
+        <v>675</v>
+      </c>
+      <c r="B776" s="2"/>
+    </row>
+    <row r="777" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A777" s="3" t="s">
         <v>676</v>
       </c>
-      <c r="B775" s="2">
-        <v>446.875</v>
-      </c>
-    </row>
-    <row r="776" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B776" s="2"/>
-    </row>
-    <row r="777" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A777" s="13" t="s">
-        <v>677</v>
-      </c>
-      <c r="B777" s="2"/>
+      <c r="B777" s="2">
+        <v>607.75</v>
+      </c>
     </row>
     <row r="778" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A778" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B778" s="2">
         <v>607.75</v>
@@ -8577,7 +8568,7 @@
     </row>
     <row r="779" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A779" s="3" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B779" s="2">
         <v>607.75</v>
@@ -8585,7 +8576,7 @@
     </row>
     <row r="780" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A780" s="3" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="B780" s="2">
         <v>607.75</v>
@@ -8593,32 +8584,32 @@
     </row>
     <row r="781" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A781" s="3" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B781" s="2">
         <v>607.75</v>
       </c>
     </row>
     <row r="782" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A782" s="3" t="s">
+      <c r="B782" s="2"/>
+    </row>
+    <row r="783" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A783" s="14" t="s">
+        <v>681</v>
+      </c>
+      <c r="B783" s="2"/>
+    </row>
+    <row r="784" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A784" s="3" t="s">
         <v>682</v>
       </c>
-      <c r="B782" s="2">
-        <v>607.75</v>
-      </c>
-    </row>
-    <row r="783" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B783" s="2"/>
-    </row>
-    <row r="784" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A784" s="13" t="s">
-        <v>683</v>
-      </c>
-      <c r="B784" s="2"/>
+      <c r="B784" s="2">
+        <v>858</v>
+      </c>
     </row>
     <row r="785" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A785" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B785" s="2">
         <v>858</v>
@@ -8626,7 +8617,7 @@
     </row>
     <row r="786" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A786" s="3" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="B786" s="2">
         <v>858</v>
@@ -8634,7 +8625,7 @@
     </row>
     <row r="787" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A787" s="3" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B787" s="2">
         <v>858</v>
@@ -8642,7 +8633,7 @@
     </row>
     <row r="788" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A788" s="3" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B788" s="2">
         <v>858</v>
@@ -8650,41 +8641,41 @@
     </row>
     <row r="789" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A789" s="3" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B789" s="2">
         <v>858</v>
       </c>
     </row>
     <row r="790" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A790" s="3" t="s">
-        <v>689</v>
-      </c>
-      <c r="B790" s="2">
-        <v>858</v>
-      </c>
+      <c r="B790" s="2"/>
     </row>
     <row r="791" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B791" s="2"/>
     </row>
     <row r="792" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A792" s="21" t="s">
+        <v>688</v>
+      </c>
       <c r="B792" s="2"/>
     </row>
     <row r="793" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A793" s="21" t="s">
+      <c r="A793" s="14" t="s">
+        <v>689</v>
+      </c>
+      <c r="B793" s="2"/>
+    </row>
+    <row r="794" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A794" s="3" t="s">
         <v>690</v>
       </c>
-      <c r="B793" s="2"/>
-    </row>
-    <row r="794" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A794" s="13" t="s">
-        <v>691</v>
-      </c>
-      <c r="B794" s="2"/>
+      <c r="B794" s="2">
+        <v>812.5</v>
+      </c>
     </row>
     <row r="795" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A795" s="3" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B795" s="2">
         <v>812.5</v>
@@ -8692,7 +8683,7 @@
     </row>
     <row r="796" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A796" s="3" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B796" s="2">
         <v>812.5</v>
@@ -8700,7 +8691,7 @@
     </row>
     <row r="797" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A797" s="3" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B797" s="2">
         <v>812.5</v>
@@ -8708,7 +8699,7 @@
     </row>
     <row r="798" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A798" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="B798" s="2">
         <v>812.5</v>
@@ -8716,7 +8707,7 @@
     </row>
     <row r="799" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A799" s="3" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B799" s="2">
         <v>812.5</v>
@@ -8724,7 +8715,7 @@
     </row>
     <row r="800" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A800" s="3" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="B800" s="2">
         <v>812.5</v>
@@ -8732,7 +8723,7 @@
     </row>
     <row r="801" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A801" s="3" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="B801" s="2">
         <v>812.5</v>
@@ -8740,7 +8731,7 @@
     </row>
     <row r="802" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A802" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="B802" s="2">
         <v>812.5</v>
@@ -8748,32 +8739,32 @@
     </row>
     <row r="803" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A803" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B803" s="2">
         <v>812.5</v>
       </c>
     </row>
     <row r="804" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A804" s="3" t="s">
+      <c r="B804" s="2"/>
+    </row>
+    <row r="805" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A805" s="14" t="s">
+        <v>369</v>
+      </c>
+      <c r="B805" s="2"/>
+    </row>
+    <row r="806" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A806" s="8" t="s">
+        <v>700</v>
+      </c>
+      <c r="B806" s="2">
+        <v>1137.5</v>
+      </c>
+    </row>
+    <row r="807" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A807" s="3" t="s">
         <v>701</v>
-      </c>
-      <c r="B804" s="2">
-        <v>812.5</v>
-      </c>
-    </row>
-    <row r="805" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B805" s="2"/>
-    </row>
-    <row r="806" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A806" s="13" t="s">
-        <v>369</v>
-      </c>
-      <c r="B806" s="2"/>
-    </row>
-    <row r="807" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A807" s="8" t="s">
-        <v>702</v>
       </c>
       <c r="B807" s="2">
         <v>1137.5</v>
@@ -8781,7 +8772,7 @@
     </row>
     <row r="808" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A808" s="3" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="B808" s="2">
         <v>1137.5</v>
@@ -8789,7 +8780,7 @@
     </row>
     <row r="809" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A809" s="3" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B809" s="2">
         <v>1137.5</v>
@@ -8797,7 +8788,7 @@
     </row>
     <row r="810" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A810" s="3" t="s">
-        <v>705</v>
+        <v>466</v>
       </c>
       <c r="B810" s="2">
         <v>1137.5</v>
@@ -8805,7 +8796,7 @@
     </row>
     <row r="811" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A811" s="3" t="s">
-        <v>466</v>
+        <v>704</v>
       </c>
       <c r="B811" s="2">
         <v>1137.5</v>
@@ -8813,7 +8804,7 @@
     </row>
     <row r="812" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A812" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B812" s="2">
         <v>1137.5</v>
@@ -8821,7 +8812,7 @@
     </row>
     <row r="813" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A813" s="3" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="B813" s="2">
         <v>1137.5</v>
@@ -8829,7 +8820,7 @@
     </row>
     <row r="814" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A814" s="3" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B814" s="2">
         <v>1137.5</v>
@@ -8837,7 +8828,7 @@
     </row>
     <row r="815" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A815" s="3" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="B815" s="2">
         <v>1137.5</v>
@@ -8845,29 +8836,29 @@
     </row>
     <row r="816" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A816" s="3" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="B816" s="2">
         <v>1137.5</v>
       </c>
     </row>
     <row r="817" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A817" s="3" t="s">
-        <v>711</v>
-      </c>
-      <c r="B817" s="2">
-        <v>1137.5</v>
-      </c>
+      <c r="A817" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="B817" s="2"/>
     </row>
     <row r="818" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A818" s="13" t="s">
-        <v>275</v>
-      </c>
-      <c r="B818" s="2"/>
+      <c r="A818" s="3" t="s">
+        <v>710</v>
+      </c>
+      <c r="B818" s="2">
+        <v>1462.5</v>
+      </c>
     </row>
     <row r="819" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A819" s="3" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B819" s="2">
         <v>1462.5</v>
@@ -8875,7 +8866,7 @@
     </row>
     <row r="820" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A820" s="3" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B820" s="2">
         <v>1462.5</v>
@@ -8883,7 +8874,7 @@
     </row>
     <row r="821" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A821" s="3" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B821" s="2">
         <v>1462.5</v>
@@ -8891,7 +8882,7 @@
     </row>
     <row r="822" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A822" s="3" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B822" s="2">
         <v>1462.5</v>
@@ -8899,7 +8890,7 @@
     </row>
     <row r="823" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A823" s="3" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B823" s="2">
         <v>1462.5</v>
@@ -8907,7 +8898,7 @@
     </row>
     <row r="824" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A824" s="3" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B824" s="2">
         <v>1462.5</v>
@@ -8915,7 +8906,7 @@
     </row>
     <row r="825" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A825" s="3" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B825" s="2">
         <v>1462.5</v>
@@ -8923,7 +8914,7 @@
     </row>
     <row r="826" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A826" s="3" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="B826" s="2">
         <v>1462.5</v>
@@ -8931,31 +8922,31 @@
     </row>
     <row r="827" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A827" s="3" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B827" s="2">
         <v>1462.5</v>
       </c>
     </row>
     <row r="828" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A828" s="3" t="s">
-        <v>721</v>
+      <c r="A828" s="14" t="s">
+        <v>382</v>
       </c>
       <c r="B828" s="2">
-        <v>1462.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="829" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A829" s="13" t="s">
-        <v>382</v>
+      <c r="A829" s="3" t="s">
+        <v>720</v>
       </c>
       <c r="B829" s="2">
-        <v>0</v>
+        <v>1727.375</v>
       </c>
     </row>
     <row r="830" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A830" s="3" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B830" s="2">
         <v>1727.375</v>
@@ -8963,31 +8954,31 @@
     </row>
     <row r="831" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A831" s="3" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B831" s="2">
         <v>1727.375</v>
       </c>
     </row>
     <row r="832" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A832" s="3" t="s">
-        <v>724</v>
+      <c r="A832" s="14" t="s">
+        <v>571</v>
       </c>
       <c r="B832" s="2">
-        <v>1727.375</v>
+        <v>0</v>
       </c>
     </row>
     <row r="833" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A833" s="13" t="s">
-        <v>572</v>
+      <c r="A833" s="3" t="s">
+        <v>723</v>
       </c>
       <c r="B833" s="2">
-        <v>0</v>
+        <v>1930.5</v>
       </c>
     </row>
     <row r="834" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A834" s="3" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="B834" s="2">
         <v>1930.5</v>
@@ -8995,7 +8986,7 @@
     </row>
     <row r="835" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A835" s="3" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B835" s="2">
         <v>1930.5</v>
@@ -9003,7 +8994,7 @@
     </row>
     <row r="836" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A836" s="3" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B836" s="2">
         <v>1930.5</v>
@@ -9011,31 +9002,31 @@
     </row>
     <row r="837" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A837" s="3" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="B837" s="2">
         <v>1930.5</v>
       </c>
     </row>
     <row r="838" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A838" s="3" t="s">
-        <v>729</v>
+      <c r="A838" s="14" t="s">
+        <v>574</v>
       </c>
       <c r="B838" s="2">
-        <v>1930.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="839" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A839" s="13" t="s">
-        <v>576</v>
+      <c r="A839" s="3" t="s">
+        <v>728</v>
       </c>
       <c r="B839" s="2">
-        <v>0</v>
+        <v>2133.625</v>
       </c>
     </row>
     <row r="840" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A840" s="3" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B840" s="2">
         <v>2133.625</v>
@@ -9043,7 +9034,7 @@
     </row>
     <row r="841" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A841" s="3" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B841" s="2">
         <v>2133.625</v>
@@ -9051,7 +9042,7 @@
     </row>
     <row r="842" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A842" s="3" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B842" s="2">
         <v>2133.625</v>
@@ -9059,7 +9050,7 @@
     </row>
     <row r="843" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A843" s="3" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B843" s="2">
         <v>2133.625</v>
@@ -9067,7 +9058,7 @@
     </row>
     <row r="844" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A844" s="3" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B844" s="2">
         <v>2133.625</v>
@@ -9075,7 +9066,7 @@
     </row>
     <row r="845" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A845" s="3" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B845" s="2">
         <v>2133.625</v>
@@ -9083,144 +9074,144 @@
     </row>
     <row r="846" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A846" s="3" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="B846" s="2">
         <v>2133.625</v>
       </c>
     </row>
     <row r="847" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A847" s="3" t="s">
-        <v>737</v>
-      </c>
       <c r="B847" s="2">
-        <v>2133.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="848" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A848" s="14" t="s">
+        <v>736</v>
+      </c>
       <c r="B848" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="849" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A849" s="13" t="s">
-        <v>738</v>
+      <c r="A849" s="3" t="s">
+        <v>737</v>
       </c>
       <c r="B849" s="2">
-        <v>0</v>
+        <v>1161.875</v>
       </c>
     </row>
     <row r="850" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A850" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="B850" s="2">
+        <v>1405.625</v>
+      </c>
+    </row>
+    <row r="851" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B851" s="2"/>
+    </row>
+    <row r="852" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A852" s="12" t="s">
+        <v>738</v>
+      </c>
+      <c r="B852" s="2"/>
+    </row>
+    <row r="853" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A853" s="3" t="s">
         <v>739</v>
       </c>
-      <c r="B850" s="2">
-        <v>1161.875</v>
-      </c>
-    </row>
-    <row r="851" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A851" s="3" t="s">
-        <v>701</v>
-      </c>
-      <c r="B851" s="2">
-        <v>1405.625</v>
-      </c>
-    </row>
-    <row r="852" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B852" s="2"/>
-    </row>
-    <row r="853" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A853" s="12" t="s">
-        <v>740</v>
-      </c>
-      <c r="B853" s="2"/>
+      <c r="B853" s="2">
+        <v>1625</v>
+      </c>
     </row>
     <row r="854" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A854" s="3" t="s">
-        <v>741</v>
+        <v>199</v>
       </c>
       <c r="B854" s="2">
-        <v>1625</v>
+        <v>2380.625</v>
       </c>
     </row>
     <row r="855" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A855" s="3" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="B855" s="2">
-        <v>2380.625</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="856" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A856" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B856" s="2">
         <v>1625</v>
       </c>
     </row>
     <row r="857" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A857" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="B857" s="2">
-        <v>1625</v>
-      </c>
+      <c r="B857" s="2"/>
     </row>
     <row r="858" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A858" s="14" t="s">
+        <v>740</v>
+      </c>
       <c r="B858" s="2"/>
     </row>
     <row r="859" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A859" s="13" t="s">
+      <c r="A859" s="3" t="s">
+        <v>741</v>
+      </c>
+      <c r="B859" s="2">
+        <v>2136.875</v>
+      </c>
+    </row>
+    <row r="860" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B860" s="2"/>
+    </row>
+    <row r="861" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A861" s="14" t="s">
         <v>742</v>
       </c>
-      <c r="B859" s="2"/>
-    </row>
-    <row r="860" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A860" s="3" t="s">
+      <c r="B861" s="2"/>
+    </row>
+    <row r="862" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A862" s="3" t="s">
         <v>743</v>
       </c>
-      <c r="B860" s="2">
-        <v>2136.875</v>
-      </c>
-    </row>
-    <row r="861" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B861" s="2"/>
-    </row>
-    <row r="862" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A862" s="13" t="s">
+      <c r="B862" s="2">
+        <v>3250</v>
+      </c>
+    </row>
+    <row r="863" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B863" s="2"/>
+    </row>
+    <row r="864" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A864" s="14" t="s">
         <v>744</v>
       </c>
-      <c r="B862" s="2"/>
-    </row>
-    <row r="863" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A863" s="3" t="s">
+      <c r="B864" s="2"/>
+    </row>
+    <row r="865" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A865" s="3" t="s">
         <v>745</v>
       </c>
-      <c r="B863" s="2">
-        <v>3250</v>
-      </c>
-    </row>
-    <row r="864" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B864" s="2"/>
-    </row>
-    <row r="865" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A865" s="13" t="s">
-        <v>746</v>
-      </c>
-      <c r="B865" s="2"/>
+      <c r="B865" s="2">
+        <v>1543.75</v>
+      </c>
     </row>
     <row r="866" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A866" s="3" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B866" s="2">
-        <v>1543.75</v>
+        <v>2136.875</v>
       </c>
     </row>
     <row r="867" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A867" s="3" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="B867" s="2">
         <v>2136.875</v>
@@ -9228,7 +9219,7 @@
     </row>
     <row r="868" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A868" s="3" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B868" s="2">
         <v>2136.875</v>
@@ -9236,7 +9227,7 @@
     </row>
     <row r="869" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A869" s="3" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B869" s="2">
         <v>2136.875</v>
@@ -9244,7 +9235,7 @@
     </row>
     <row r="870" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A870" s="3" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B870" s="2">
         <v>2136.875</v>
@@ -9252,7 +9243,7 @@
     </row>
     <row r="871" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A871" s="3" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B871" s="2">
         <v>2136.875</v>
@@ -9260,64 +9251,56 @@
     </row>
     <row r="872" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A872" s="3" t="s">
-        <v>753</v>
+        <v>732</v>
       </c>
       <c r="B872" s="2">
         <v>2136.875</v>
       </c>
     </row>
     <row r="873" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A873" s="3" t="s">
-        <v>734</v>
-      </c>
-      <c r="B873" s="2">
-        <v>2136.875</v>
-      </c>
+      <c r="B873" s="2"/>
     </row>
     <row r="874" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A874" s="14" t="s">
+        <v>752</v>
+      </c>
       <c r="B874" s="2"/>
     </row>
     <row r="875" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A875" s="13" t="s">
+      <c r="A875" s="3" t="s">
+        <v>753</v>
+      </c>
+      <c r="B875" s="2">
+        <v>2372.5</v>
+      </c>
+    </row>
+    <row r="876" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B876" s="2"/>
+    </row>
+    <row r="877" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A877" s="14" t="s">
         <v>754</v>
       </c>
-      <c r="B875" s="2"/>
-    </row>
-    <row r="876" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A876" s="3" t="s">
+      <c r="B877" s="2"/>
+    </row>
+    <row r="878" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A878" s="3" t="s">
         <v>755</v>
       </c>
-      <c r="B876" s="2">
-        <v>2372.5</v>
-      </c>
-    </row>
-    <row r="877" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B877" s="2"/>
-    </row>
-    <row r="878" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A878" s="13" t="s">
-        <v>756</v>
-      </c>
-      <c r="B878" s="2"/>
+      <c r="B878" s="2">
+        <v>2031.25</v>
+      </c>
     </row>
     <row r="879" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A879" s="3" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B879" s="2">
-        <v>2031.25</v>
+        <v>1283.75</v>
       </c>
     </row>
     <row r="880" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A880" s="3" t="s">
-        <v>758</v>
-      </c>
-      <c r="B880" s="2">
-        <v>1283.75</v>
-      </c>
-    </row>
-    <row r="881" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B881" s="2"/>
+      <c r="B880" s="2"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" gridLines="1"/>

</xml_diff>